<commit_message>
Improvements in capture+graph merge logic and tree_perf (#161)
* Improved logic for capture roots

* fixed a bug in unified perf report

* modified UIDs for synthetic events

* reformattingh

* fixing regression tests, main difference is in UIDs for inference

* modified perf report based on tree_perf changes

---------

Co-authored-by: Deval Shah <devashah@amd.com>
</commit_message>
<xml_diff>
--- a/tests/traces/inference/graph_full/perf_report.xlsx
+++ b/tests/traces/inference/graph_full/perf_report.xlsx
@@ -1298,7 +1298,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>{'elementwise', 'other'}</t>
+          <t>{'other', 'elementwise'}</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1638,7 +1638,7 @@
         <v>7171.5322265625</v>
       </c>
       <c r="O2" t="n">
-        <v>3436</v>
+        <v>3437</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -1720,7 +1720,7 @@
         <v>724.361328125</v>
       </c>
       <c r="O3" t="n">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -1802,7 +1802,7 @@
         <v>387.01171875</v>
       </c>
       <c r="O4" t="n">
-        <v>2402</v>
+        <v>2403</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         <v>375.1181640625</v>
       </c>
       <c r="O5" t="n">
-        <v>3909</v>
+        <v>3910</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         <v>366.2138671875</v>
       </c>
       <c r="O6" t="n">
-        <v>3313</v>
+        <v>3314</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
         <v>292.3740234375</v>
       </c>
       <c r="O7" t="n">
-        <v>7472</v>
+        <v>7473</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -2210,7 +2210,7 @@
         <v>200.65234375</v>
       </c>
       <c r="O9" t="n">
-        <v>3403</v>
+        <v>3404</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -2292,7 +2292,7 @@
         <v>170.900390625</v>
       </c>
       <c r="O10" t="n">
-        <v>3341</v>
+        <v>3342</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -2374,7 +2374,7 @@
         <v>155.1376953125</v>
       </c>
       <c r="O11" t="n">
-        <v>7386</v>
+        <v>7387</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -2456,7 +2456,7 @@
         <v>149.73828125</v>
       </c>
       <c r="O12" t="n">
-        <v>2414</v>
+        <v>2415</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -2538,7 +2538,7 @@
         <v>136.41015625</v>
       </c>
       <c r="O13" t="n">
-        <v>2527</v>
+        <v>2528</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -2620,7 +2620,7 @@
         <v>122.6103515625</v>
       </c>
       <c r="O14" t="n">
-        <v>3426</v>
+        <v>3427</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -2702,7 +2702,7 @@
         <v>119.814453125</v>
       </c>
       <c r="O15" t="n">
-        <v>3502</v>
+        <v>3503</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -2864,7 +2864,7 @@
         <v>10.59765625</v>
       </c>
       <c r="O17" t="n">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
@@ -3026,7 +3026,7 @@
         <v>5.9990234375</v>
       </c>
       <c r="O19" t="n">
-        <v>2339</v>
+        <v>2340</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -3888,7 +3888,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>127697</v>
+        <v>127709</v>
       </c>
       <c r="K2" t="n">
         <v>24</v>
@@ -4035,7 +4035,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>127696</v>
+        <v>127708</v>
       </c>
       <c r="K3" t="n">
         <v>24</v>
@@ -4182,7 +4182,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="K4" t="n">
         <v>24</v>
@@ -4339,7 +4339,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2360</v>
+        <v>2361</v>
       </c>
       <c r="K5" t="n">
         <v>24</v>
@@ -4496,7 +4496,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3909</v>
+        <v>3910</v>
       </c>
       <c r="K6" t="n">
         <v>24</v>
@@ -4619,7 +4619,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>3271</v>
+        <v>3272</v>
       </c>
       <c r="K7" t="n">
         <v>24</v>
@@ -4776,7 +4776,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>7472</v>
+        <v>7473</v>
       </c>
       <c r="K8" t="n">
         <v>23</v>
@@ -5048,7 +5048,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>3361</v>
+        <v>3362</v>
       </c>
       <c r="K10" t="n">
         <v>24</v>
@@ -5205,7 +5205,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>3341</v>
+        <v>3342</v>
       </c>
       <c r="K11" t="n">
         <v>24</v>
@@ -5328,7 +5328,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>7386</v>
+        <v>7387</v>
       </c>
       <c r="K12" t="n">
         <v>24</v>
@@ -5451,7 +5451,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>2414</v>
+        <v>2415</v>
       </c>
       <c r="K13" t="n">
         <v>24</v>
@@ -5574,7 +5574,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>127698</v>
+        <v>127710</v>
       </c>
       <c r="K14" t="n">
         <v>24</v>
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>2527</v>
+        <v>2528</v>
       </c>
       <c r="K15" t="n">
         <v>24</v>
@@ -5810,7 +5810,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>3426</v>
+        <v>3427</v>
       </c>
       <c r="K16" t="n">
         <v>24</v>
@@ -5933,7 +5933,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>3502</v>
+        <v>3503</v>
       </c>
       <c r="K17" t="n">
         <v>24</v>
@@ -6209,7 +6209,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="K19" t="n">
         <v>1</v>
@@ -6467,7 +6467,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>2339</v>
+        <v>2340</v>
       </c>
       <c r="K21" t="n">
         <v>1</v>
@@ -7702,7 +7702,7 @@
         <v>24</v>
       </c>
       <c r="AP2" t="n">
-        <v>2360</v>
+        <v>2361</v>
       </c>
     </row>
     <row r="3">
@@ -7872,7 +7872,7 @@
         <v>24</v>
       </c>
       <c r="AP3" t="n">
-        <v>2402</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="4">
@@ -8042,7 +8042,7 @@
         <v>24</v>
       </c>
       <c r="AP4" t="n">
-        <v>3271</v>
+        <v>3272</v>
       </c>
     </row>
     <row r="5">
@@ -8212,7 +8212,7 @@
         <v>24</v>
       </c>
       <c r="AP5" t="n">
-        <v>3313</v>
+        <v>3314</v>
       </c>
     </row>
     <row r="6">
@@ -8710,7 +8710,7 @@
         <v>24</v>
       </c>
       <c r="AP8" t="n">
-        <v>3361</v>
+        <v>3362</v>
       </c>
     </row>
     <row r="9">
@@ -8880,7 +8880,7 @@
         <v>24</v>
       </c>
       <c r="AP9" t="n">
-        <v>3403</v>
+        <v>3404</v>
       </c>
     </row>
   </sheetData>
@@ -9266,7 +9266,7 @@
         <v>24</v>
       </c>
       <c r="AO2" t="n">
-        <v>127697</v>
+        <v>127709</v>
       </c>
     </row>
     <row r="3">
@@ -9431,7 +9431,7 @@
         <v>24</v>
       </c>
       <c r="AO3" t="n">
-        <v>127696</v>
+        <v>127708</v>
       </c>
     </row>
   </sheetData>
@@ -9927,7 +9927,7 @@
         <v>12</v>
       </c>
       <c r="AZ2" t="n">
-        <v>7603</v>
+        <v>7604</v>
       </c>
     </row>
     <row r="3">
@@ -10147,7 +10147,7 @@
         <v>12</v>
       </c>
       <c r="AZ3" t="n">
-        <v>2533</v>
+        <v>2534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>